<commit_message>
nang cap vione platform
</commit_message>
<xml_diff>
--- a/apps/vione_app_fe/public/docs/TIEN_DO_CONG_VIEC_HE_THONG_VA_APP_VIONE.xlsx
+++ b/apps/vione_app_fe/public/docs/TIEN_DO_CONG_VIEC_HE_THONG_VA_APP_VIONE.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="151">
   <si>
     <t>Mã WBS</t>
   </si>
@@ -308,13 +308,169 @@
   </si>
   <si>
     <t>Technical Writer &amp; BA</t>
+  </si>
+  <si>
+    <t>5.0</t>
+  </si>
+  <si>
+    <t>Full-Stack (BE / Web CRM / Mobile)</t>
+  </si>
+  <si>
+    <t>Phân Quyền Phòng Ban Chuyên Trách (Department-based RBAC)</t>
+  </si>
+  <si>
+    <t>Khối -&gt; Phòng ban -&gt; Nhóm chuyên trách (vione_community_departments). Kiểm soát 5 cờ quyền: canAssign, canAccept, canReport, canHandover, canMeet. Department Guard bảo mật dữ liệu theo phòng ban.</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>Solution Architect &amp; Fullstack Lead</t>
+  </si>
+  <si>
+    <t>03/10/2026</t>
+  </si>
+  <si>
+    <t>07/10/2026</t>
+  </si>
+  <si>
+    <t>Department RBAC Engine, Department Guard, DepartmentPermissionsModal, RESTful APIs /department-members</t>
+  </si>
+  <si>
+    <t>5.1</t>
+  </si>
+  <si>
+    <t>Full-Stack (NestJS BE / CRM / App)</t>
+  </si>
+  <si>
+    <t>Cơ Chế Bàn Giao Công Việc Tự Động (Auto-Handover Engine)</t>
+  </si>
+  <si>
+    <t>Gom và chuyển giao hàng loạt công việc (tasks), khách hàng (CRM customers), cơ hội (deals) khi luân chuyển hoặc thôi việc. Tự động sinh biên bản bàn giao, phát thông báo Push/In-app, lưu vết audit trail handover_history.</t>
+  </si>
+  <si>
+    <t>Senior Backend Dev &amp; Mobile Lead</t>
+  </si>
+  <si>
+    <t>05/10/2026</t>
+  </si>
+  <si>
+    <t>08/10/2026</t>
+  </si>
+  <si>
+    <t>Auto-Handover Service, Bulk Reassignment UI, Handover History Audit Trail, Notification Push</t>
+  </si>
+  <si>
+    <t>5.2</t>
+  </si>
+  <si>
+    <t>Full-Stack (Web CRM &amp; Mobile App)</t>
+  </si>
+  <si>
+    <t>Mô Hình Cộng Đồng Hợp Nhất &amp; Gói Dùng Thử 30 Ngày (Unified Community &amp; 30-Day Subscription)</t>
+  </si>
+  <si>
+    <t>Hợp nhất 2 mô hình cộng đồng (Nội bộ &amp; B2B) thành 1 mô hình toàn năng duy nhất (tasks, supervision, opportunities, news, events, members). Gating phân hệ giao việc tại Trang chủ (chỉ hiện khi có gói hoặc dùng thử 30 ngày free). Thẻ CTA Champagne Gold và form khởi tạo 1-chạm.</t>
+  </si>
+  <si>
+    <t>Product Owner &amp; Frontend Lead</t>
+  </si>
+  <si>
+    <t>10/10/2026</t>
+  </si>
+  <si>
+    <t>Unified Community Model, Subscription Trial Gating, CommunityPackageTrialCta, CreateCommunityGroupModal</t>
+  </si>
+  <si>
+    <t>5.3</t>
+  </si>
+  <si>
+    <t>Full-Stack (WebRTC / Mobile / Web)</t>
+  </si>
+  <si>
+    <t>Họp Ban Trực Tuyến 1-Chạm (Instant Department Meeting - C-Level Room)</t>
+  </si>
+  <si>
+    <t>Nút họp ban 1-chạm mạ vàng trên thanh công cụ điều hành công việc. Khởi tạo tức thì phòng họp WebRTC C-Level bảo mật cao, tự động gửi thông báo triệu tập khẩn cấp đến nhân sự phòng ban.</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>Mobile Dev &amp; WebRTC Engineer</t>
+  </si>
+  <si>
+    <t>11/10/2026</t>
+  </si>
+  <si>
+    <t>Instant Meeting Trigger, C-Level Executive Room WebRTC, Urgent Push Notification</t>
+  </si>
+  <si>
+    <t>5.4</t>
+  </si>
+  <si>
+    <t>Full-Stack (Office Document Parser)</t>
+  </si>
+  <si>
+    <t>Import &amp; Export Đa Định Dạng (Excel &amp; Word for Assigner &amp; Assignee)</t>
+  </si>
+  <si>
+    <t>Người giao việc: Nạp công việc hàng loạt từ tệp .xlsx/.csv và đề án nhiệm vụ từ .docx. Người nhận việc: Đính kèm đồng thời báo cáo Word và bảng tính số liệu Excel khi nghiệm thu công việc.</t>
+  </si>
+  <si>
+    <t>Backend &amp; Frontend Dev</t>
+  </si>
+  <si>
+    <t>09/10/2026</t>
+  </si>
+  <si>
+    <t>Excel Bulk Task Importer, Word Scheme Parser, Dual Word/Excel Proof Attachment Modal</t>
+  </si>
+  <si>
+    <t>5.5</t>
+  </si>
+  <si>
+    <t>Web CRM ViOne Platform</t>
+  </si>
+  <si>
+    <t>Màn Đăng Nhập CRM Tĩnh C-Level &amp; Bộ Lọc Trạng Thái Toàn Diện (Dashboard &amp; Marketplace)</t>
+  </si>
+  <si>
+    <t>Triệt tiêu 100% animation xoay vòng gây phân tâm, áp dụng kiến trúc tĩnh 2 cột mạ vàng sang trọng. Trang bị bộ lọc trạng thái đa chiều (Status Filter Tabs) kèm badge đếm số lượng thời gian thực trên C-Level Dashboard và Sàn Marketplace.</t>
+  </si>
+  <si>
+    <t>UI/UX Lead &amp; Senior Frontend Dev</t>
+  </si>
+  <si>
+    <t>12/10/2026</t>
+  </si>
+  <si>
+    <t>Static C-Level Auth Screen (/auth), ExecutiveDashboard Status Filters, Marketplace Category Filters</t>
+  </si>
+  <si>
+    <t>5.6</t>
+  </si>
+  <si>
+    <t>Mobile Native App &amp; PWA (/connect-app)</t>
+  </si>
+  <si>
+    <t>Đồng Bộ Hoàn Toàn Chức Năng ViOne PWA Với ViOne Native App &amp; Cân Đối UI/UX</t>
+  </si>
+  <si>
+    <t>Đồng bộ 100% tính năng giữa PWA (/connect-app) và Native App (apps/mobile_vione). Cân đối chuẩn xác bố trí text, icon, typography, safe area insets (Dynamic Island / Gesture Nav) trên 4 tabs chính (Home, Network, Community, Me), nút V trung tâm (VActionSheet), PostMomentModal, CardScanReviewModal, ViOneVoiceAssistantModal.</t>
+  </si>
+  <si>
+    <t>Mobile Lead &amp; Senior UI/UX Designer</t>
+  </si>
+  <si>
+    <t>100% PWA-Native Parity, CustomBottomTabBar Insets Alignment, Balanced Mobile Native Layout</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -338,6 +494,17 @@
       <sz val="10"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <color rgb="000000"/>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="10B981"/>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -352,7 +519,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -375,11 +542,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="E2E8F0"/>
+      </left>
+      <right style="thin">
+        <color rgb="E2E8F0"/>
+      </right>
+      <top style="thin">
+        <color rgb="E2E8F0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="E2E8F0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -397,6 +579,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -738,7 +929,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K19"/>
+  <dimension ref="A1:K26"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1239,8 +1430,253 @@
         <v>17</v>
       </c>
     </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A20" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="B20" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="C20" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="D20" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="E20" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="F20" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="G20" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="H20" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="I20" s="7">
+        <v>100</v>
+      </c>
+      <c r="J20" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="K20" s="8" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A21" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="B21" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="C21" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="D21" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="E21" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="F21" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="G21" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="H21" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="I21" s="7">
+        <v>100</v>
+      </c>
+      <c r="J21" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="K21" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A22" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="D22" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="E22" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="F22" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="G22" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="H22" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="I22" s="7">
+        <v>100</v>
+      </c>
+      <c r="J22" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="K22" s="8" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A23" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="B23" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="C23" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="D23" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="E23" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="F23" s="8" t="s">
+        <v>128</v>
+      </c>
+      <c r="G23" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="H23" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="I23" s="7">
+        <v>100</v>
+      </c>
+      <c r="J23" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="K23" s="8" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A24" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>132</v>
+      </c>
+      <c r="C24" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="D24" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="E24" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="F24" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="G24" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="H24" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="I24" s="7">
+        <v>100</v>
+      </c>
+      <c r="J24" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="K24" s="8" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A25" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="B25" s="8" t="s">
+        <v>139</v>
+      </c>
+      <c r="C25" s="8" t="s">
+        <v>140</v>
+      </c>
+      <c r="D25" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="E25" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="F25" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="G25" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="H25" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="I25" s="7">
+        <v>100</v>
+      </c>
+      <c r="J25" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="K25" s="8" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A26" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="B26" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="C26" s="8" t="s">
+        <v>147</v>
+      </c>
+      <c r="D26" s="8" t="s">
+        <v>148</v>
+      </c>
+      <c r="E26" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="F26" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="G26" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="H26" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="I26" s="7">
+        <v>100</v>
+      </c>
+      <c r="J26" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="K26" s="8" t="s">
+        <v>150</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>